<commit_message>
Add WeMath and VLMBias LLM extraction scores
</commit_message>
<xml_diff>
--- a/results/qwen25vl7b_candidate23_1000_judge_usage_summary.xlsx
+++ b/results/qwen25vl7b_candidate23_1000_judge_usage_summary.xlsx
@@ -458,12 +458,12 @@
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="40" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="20" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="19" customWidth="1" min="6" max="6"/>
+    <col width="19" customWidth="1" min="7" max="7"/>
     <col width="21" customWidth="1" min="8" max="8"/>
-    <col width="20" customWidth="1" min="9" max="9"/>
-    <col width="20" customWidth="1" min="10" max="10"/>
-    <col width="21" customWidth="1" min="11" max="11"/>
+    <col width="19" customWidth="1" min="9" max="9"/>
+    <col width="19" customWidth="1" min="10" max="10"/>
+    <col width="20" customWidth="1" min="11" max="11"/>
     <col width="28" customWidth="1" min="12" max="12"/>
     <col width="31" customWidth="1" min="13" max="13"/>
     <col width="40" customWidth="1" min="14" max="14"/>
@@ -886,31 +886,19 @@
       <c r="P4" t="n">
         <v>127.657</v>
       </c>
-      <c r="Q4" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
+      <c r="Q4" t="inlineStr"/>
       <c r="R4" t="inlineStr">
         <is>
           <t>Deterministic point/region hit</t>
         </is>
       </c>
-      <c r="S4" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
+      <c r="S4" t="inlineStr"/>
       <c r="T4" t="inlineStr">
         <is>
           <t>Deterministic point/region hit</t>
         </is>
       </c>
-      <c r="U4" s="3" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
+      <c r="U4" s="3" t="inlineStr"/>
       <c r="V4" t="inlineStr">
         <is>
           <t>VLMEvalKit ScreenSpot deterministic localization scorer.</t>
@@ -994,31 +982,19 @@
       <c r="P5" t="n">
         <v>184.412</v>
       </c>
-      <c r="Q5" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
+      <c r="Q5" t="inlineStr"/>
       <c r="R5" t="inlineStr">
         <is>
           <t>Deterministic point/region hit</t>
         </is>
       </c>
-      <c r="S5" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
+      <c r="S5" t="inlineStr"/>
       <c r="T5" t="inlineStr">
         <is>
           <t>Deterministic point/region hit</t>
         </is>
       </c>
-      <c r="U5" s="3" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
+      <c r="U5" s="3" t="inlineStr"/>
       <c r="V5" t="inlineStr">
         <is>
           <t>VLMEvalKit ScreenSpot-Pro deterministic localization scorer.</t>
@@ -1617,23 +1593,23 @@
         <v>4.600000000000009</v>
       </c>
       <c r="I11" s="3" t="n">
-        <v>62.3</v>
+        <v>62.5</v>
       </c>
       <c r="J11" s="3" t="n">
-        <v>66.90000000000001</v>
+        <v>68</v>
       </c>
       <c r="K11" s="3" t="n">
-        <v>4.600000000000009</v>
+        <v>5.5</v>
       </c>
       <c r="L11" t="n">
-        <v>0</v>
+        <v>0.2000000000000028</v>
       </c>
       <c r="M11" t="n">
-        <v>0</v>
+        <v>1.099999999999994</v>
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>Original benchmark/local scorer</t>
+          <t>Qwen3-32B LLM extraction rescore</t>
         </is>
       </c>
       <c r="O11" t="n">
@@ -1654,7 +1630,7 @@
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>Rule option extractor</t>
+          <t>Qwen3-32B extractor</t>
         </is>
       </c>
       <c r="T11" t="inlineStr">
@@ -1664,22 +1640,22 @@
       </c>
       <c r="U11" s="3" t="inlineStr">
         <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="V11" t="inlineStr">
-        <is>
-          <t>TRACE subset-safe WeMath option-letter exact scorer.</t>
+          <t>Extraction only</t>
+        </is>
+      </c>
+      <c r="V11" s="4" t="inlineStr">
+        <is>
+          <t>Qwen3 extracts final option letter from CoT response; exact option scoring.</t>
         </is>
       </c>
       <c r="W11" s="3" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>No</t>
         </is>
       </c>
       <c r="X11" s="4" t="inlineStr">
         <is>
-          <t>Consider Qwen3 extraction-only rescore. CoT responses can bury the final option, but scoring should remain exact after extraction.</t>
+          <t>Use Qwen3 extraction plus exact option scoring; full judge is not needed for MCQ.</t>
         </is>
       </c>
       <c r="Y11" s="4" t="inlineStr">
@@ -3037,7 +3013,7 @@
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>Original benchmark/local scorer</t>
+          <t>Qwen3-32B LLM extraction rescore</t>
         </is>
       </c>
       <c r="O24" t="n">
@@ -3058,32 +3034,32 @@
       </c>
       <c r="S24" t="inlineStr">
         <is>
-          <t>Rule brace/exact extractor</t>
+          <t>Qwen3-32B braced-answer extractor</t>
         </is>
       </c>
       <c r="T24" t="inlineStr">
         <is>
-          <t>Exact match</t>
+          <t>Exact normalized match</t>
         </is>
       </c>
       <c r="U24" s="3" t="inlineStr">
         <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="V24" t="inlineStr">
-        <is>
-          <t>Local brace/exact scorer.</t>
+          <t>Extraction only</t>
+        </is>
+      </c>
+      <c r="V24" s="4" t="inlineStr">
+        <is>
+          <t>Qwen3 extracts final braced answer value; exact normalized scoring.</t>
         </is>
       </c>
       <c r="W24" s="3" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>No</t>
         </is>
       </c>
       <c r="X24" s="4" t="inlineStr">
         <is>
-          <t>Probably keep as-is; responses are very short. Consider Qwen3 extraction only if audit shows formatting drift.</t>
+          <t>Qwen3 extraction matches the original overall score; keep exact scoring and do not use full judge as primary.</t>
         </is>
       </c>
       <c r="Y24" t="inlineStr">
@@ -3115,9 +3091,9 @@
     <col width="10" customWidth="1" min="2" max="2"/>
     <col width="20" customWidth="1" min="3" max="3"/>
     <col width="19" customWidth="1" min="4" max="4"/>
-    <col width="21" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
     <col width="20" customWidth="1" min="6" max="6"/>
-    <col width="19" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
     <col width="20" customWidth="1" min="8" max="8"/>
     <col width="35" customWidth="1" min="9" max="9"/>
   </cols>
@@ -3185,19 +3161,19 @@
         <v>42.4696451402259</v>
       </c>
       <c r="E2" t="n">
-        <v>0.0615306001026634</v>
+        <v>0.06153060010266356</v>
       </c>
       <c r="F2" t="n">
-        <v>43.73585824454275</v>
+        <v>43.74455389671667</v>
       </c>
       <c r="G2" t="n">
-        <v>46.58792683993048</v>
+        <v>46.635752926887</v>
       </c>
       <c r="H2" t="n">
-        <v>2.852068595387736</v>
+        <v>2.891199030170344</v>
       </c>
       <c r="I2" t="n">
-        <v>2.790537995285073</v>
+        <v>2.829668430067681</v>
       </c>
     </row>
     <row r="3">
@@ -3216,19 +3192,19 @@
         <v>40.34226192259231</v>
       </c>
       <c r="E3" t="n">
-        <v>0.1365140542683725</v>
+        <v>0.1365140542683727</v>
       </c>
       <c r="F3" t="n">
-        <v>41.64955400480734</v>
+        <v>41.65969702134046</v>
       </c>
       <c r="G3" t="n">
-        <v>44.92408291501944</v>
+        <v>44.97986950595158</v>
       </c>
       <c r="H3" t="n">
-        <v>3.27452891021211</v>
+        <v>3.320172484611136</v>
       </c>
       <c r="I3" t="n">
-        <v>3.138014855943738</v>
+        <v>3.183658430342764</v>
       </c>
     </row>
   </sheetData>
@@ -3248,7 +3224,7 @@
     <col width="21" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="21" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3312,45 +3288,41 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="C4" t="n">
-        <v>11930</v>
+        <v>13930</v>
       </c>
       <c r="D4" t="n">
-        <v>2.727249680440551</v>
+        <v>2.876985012153428</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Scoring only</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C5" t="n">
-        <v>4000</v>
+        <v>1000</v>
       </c>
       <c r="D5" t="n">
-        <v>2.925000000000002</v>
+        <v>6.000000000000004</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Scoring only</t>
-        </is>
-      </c>
+      <c r="A6" t="inlineStr"/>
       <c r="B6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C6" t="n">
-        <v>1000</v>
+        <v>2000</v>
       </c>
       <c r="D6" t="n">
-        <v>6.000000000000004</v>
+        <v>2.300000000000001</v>
       </c>
     </row>
   </sheetData>

</xml_diff>